<commit_message>
Add PiN step 1 hybrid for Somalia___SOM
</commit_message>
<xml_diff>
--- a/platform_PiN_output/Somalia___SOM/PiN_step1_Somalia___SOM_1008_02AM.xlsx
+++ b/platform_PiN_output/Somalia___SOM/PiN_step1_Somalia___SOM_1008_02AM.xlsx
@@ -1226,10 +1226,10 @@
         <v>193260</v>
       </c>
       <c r="D3" s="33" t="n">
-        <v>59.6</v>
+        <v>59.3</v>
       </c>
       <c r="E3" s="33" t="n">
-        <v>115163</v>
+        <v>114512</v>
       </c>
       <c r="F3" s="33" t="n">
         <v>36.2</v>
@@ -1238,22 +1238,22 @@
         <v>69967</v>
       </c>
       <c r="H3" s="33" t="n">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="I3" s="33" t="n">
-        <v>7478</v>
+        <v>7413</v>
       </c>
       <c r="J3" s="33" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="K3" s="33" t="n">
-        <v>651</v>
+        <v>1367</v>
       </c>
       <c r="L3" s="33" t="n">
-        <v>40.4</v>
+        <v>40.7</v>
       </c>
       <c r="M3" s="33" t="n">
-        <v>78097</v>
+        <v>78748</v>
       </c>
       <c r="N3" s="34" t="inlineStr">
         <is>
@@ -1488,34 +1488,34 @@
         <v>25030</v>
       </c>
       <c r="D4" s="33" t="n">
-        <v>46.9</v>
+        <v>46.2</v>
       </c>
       <c r="E4" s="33" t="n">
-        <v>11741</v>
+        <v>11559</v>
       </c>
       <c r="F4" s="33" t="n">
-        <v>40</v>
+        <v>33.8</v>
       </c>
       <c r="G4" s="33" t="n">
-        <v>10012</v>
+        <v>8465</v>
       </c>
       <c r="H4" s="33" t="n">
-        <v>13.1</v>
+        <v>8</v>
       </c>
       <c r="I4" s="33" t="n">
-        <v>3277</v>
+        <v>2002</v>
       </c>
       <c r="J4" s="33" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K4" s="33" t="n">
-        <v>0</v>
+        <v>3004</v>
       </c>
       <c r="L4" s="33" t="n">
-        <v>53.1</v>
+        <v>53.8</v>
       </c>
       <c r="M4" s="33" t="n">
-        <v>13289</v>
+        <v>13471</v>
       </c>
       <c r="N4" s="34" t="inlineStr">
         <is>
@@ -2274,10 +2274,10 @@
         <v>468154</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>76</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>355672</v>
+        <v>355499</v>
       </c>
       <c r="F7" s="33" t="n">
         <v>23</v>
@@ -2295,13 +2295,13 @@
         <v>0</v>
       </c>
       <c r="K7" s="33" t="n">
-        <v>0</v>
+        <v>174</v>
       </c>
       <c r="L7" s="33" t="n">
-        <v>24</v>
+        <v>24.1</v>
       </c>
       <c r="M7" s="33" t="n">
-        <v>112482</v>
+        <v>112655</v>
       </c>
       <c r="N7" s="34" t="inlineStr">
         <is>
@@ -2830,16 +2830,16 @@
         <v>30253</v>
       </c>
       <c r="H9" s="33" t="n">
-        <v>5.3</v>
+        <v>2.6</v>
       </c>
       <c r="I9" s="33" t="n">
-        <v>4973</v>
+        <v>2487</v>
       </c>
       <c r="J9" s="33" t="n">
-        <v>0</v>
+        <v>2.6</v>
       </c>
       <c r="K9" s="33" t="n">
-        <v>0</v>
+        <v>2487</v>
       </c>
       <c r="L9" s="33" t="n">
         <v>37.4</v>
@@ -3374,16 +3374,16 @@
         <v>14809</v>
       </c>
       <c r="H11" s="33" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="I11" s="33" t="n">
-        <v>793</v>
+        <v>529</v>
       </c>
       <c r="J11" s="33" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="K11" s="33" t="n">
-        <v>0</v>
+        <v>264</v>
       </c>
       <c r="L11" s="33" t="n">
         <v>38.8</v>
@@ -4168,10 +4168,10 @@
         <v>118269</v>
       </c>
       <c r="D14" s="33" t="n">
-        <v>58</v>
+        <v>57.5</v>
       </c>
       <c r="E14" s="33" t="n">
-        <v>68582</v>
+        <v>68036</v>
       </c>
       <c r="F14" s="33" t="n">
         <v>37.8</v>
@@ -4186,16 +4186,16 @@
         <v>4998</v>
       </c>
       <c r="J14" s="33" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K14" s="33" t="n">
-        <v>0</v>
+        <v>547</v>
       </c>
       <c r="L14" s="33" t="n">
-        <v>42</v>
+        <v>42.5</v>
       </c>
       <c r="M14" s="33" t="n">
-        <v>49687</v>
+        <v>50233</v>
       </c>
       <c r="N14" s="34" t="inlineStr">
         <is>
@@ -4966,16 +4966,16 @@
         <v>26376</v>
       </c>
       <c r="H17" s="33" t="n">
-        <v>11.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I17" s="33" t="n">
-        <v>4793</v>
+        <v>3964</v>
       </c>
       <c r="J17" s="33" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="K17" s="33" t="n">
-        <v>0</v>
+        <v>829</v>
       </c>
       <c r="L17" s="33" t="n">
         <v>72.59999999999999</v>
@@ -5216,34 +5216,34 @@
         <v>79416</v>
       </c>
       <c r="D18" s="33" t="n">
-        <v>63.2</v>
+        <v>62.7</v>
       </c>
       <c r="E18" s="33" t="n">
-        <v>50215</v>
+        <v>49816</v>
       </c>
       <c r="F18" s="33" t="n">
-        <v>27.7</v>
+        <v>27.3</v>
       </c>
       <c r="G18" s="33" t="n">
-        <v>22033</v>
+        <v>21675</v>
       </c>
       <c r="H18" s="33" t="n">
-        <v>9</v>
+        <v>7.6</v>
       </c>
       <c r="I18" s="33" t="n">
-        <v>7168</v>
+        <v>6012</v>
       </c>
       <c r="J18" s="33" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="K18" s="33" t="n">
-        <v>0</v>
+        <v>1913</v>
       </c>
       <c r="L18" s="33" t="n">
-        <v>36.8</v>
+        <v>37.3</v>
       </c>
       <c r="M18" s="33" t="n">
-        <v>29201</v>
+        <v>29600</v>
       </c>
       <c r="N18" s="34" t="inlineStr">
         <is>
@@ -5478,10 +5478,10 @@
         <v>41626</v>
       </c>
       <c r="D19" s="33" t="n">
-        <v>80.59999999999999</v>
+        <v>79.3</v>
       </c>
       <c r="E19" s="33" t="n">
-        <v>33534</v>
+        <v>33000</v>
       </c>
       <c r="F19" s="33" t="n">
         <v>14.6</v>
@@ -5490,26 +5490,26 @@
         <v>6070</v>
       </c>
       <c r="H19" s="33" t="n">
-        <v>4.9</v>
+        <v>2.3</v>
       </c>
       <c r="I19" s="33" t="n">
-        <v>2022</v>
+        <v>955</v>
       </c>
       <c r="J19" s="33" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="K19" s="33" t="n">
-        <v>0</v>
+        <v>1601</v>
       </c>
       <c r="L19" s="33" t="n">
-        <v>19.4</v>
+        <v>20.7</v>
       </c>
       <c r="M19" s="33" t="n">
-        <v>8092</v>
+        <v>8626</v>
       </c>
       <c r="N19" s="34" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="O19" s="35" t="n">
@@ -5740,34 +5740,34 @@
         <v>70922</v>
       </c>
       <c r="D20" s="33" t="n">
-        <v>16.2</v>
+        <v>15.7</v>
       </c>
       <c r="E20" s="33" t="n">
-        <v>11497</v>
+        <v>11101</v>
       </c>
       <c r="F20" s="33" t="n">
-        <v>71.40000000000001</v>
+        <v>70.8</v>
       </c>
       <c r="G20" s="33" t="n">
-        <v>50620</v>
+        <v>50224</v>
       </c>
       <c r="H20" s="33" t="n">
-        <v>12.4</v>
+        <v>9</v>
       </c>
       <c r="I20" s="33" t="n">
-        <v>8804</v>
+        <v>6374</v>
       </c>
       <c r="J20" s="33" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="K20" s="33" t="n">
-        <v>0</v>
+        <v>3222</v>
       </c>
       <c r="L20" s="33" t="n">
-        <v>83.8</v>
+        <v>84.3</v>
       </c>
       <c r="M20" s="33" t="n">
-        <v>59425</v>
+        <v>59821</v>
       </c>
       <c r="N20" s="34" t="inlineStr">
         <is>
@@ -6002,10 +6002,10 @@
         <v>357720</v>
       </c>
       <c r="D21" s="33" t="n">
-        <v>46.7</v>
+        <v>45.2</v>
       </c>
       <c r="E21" s="33" t="n">
-        <v>167134</v>
+        <v>161531</v>
       </c>
       <c r="F21" s="33" t="n">
         <v>50.1</v>
@@ -6014,22 +6014,22 @@
         <v>179350</v>
       </c>
       <c r="H21" s="33" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="I21" s="33" t="n">
-        <v>11236</v>
+        <v>10451</v>
       </c>
       <c r="J21" s="33" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="K21" s="33" t="n">
-        <v>0</v>
+        <v>6388</v>
       </c>
       <c r="L21" s="33" t="n">
-        <v>53.3</v>
+        <v>54.8</v>
       </c>
       <c r="M21" s="33" t="n">
-        <v>190586</v>
+        <v>196189</v>
       </c>
       <c r="N21" s="34" t="inlineStr">
         <is>
@@ -6264,10 +6264,10 @@
         <v>22612</v>
       </c>
       <c r="D22" s="33" t="n">
-        <v>65.8</v>
+        <v>65.2</v>
       </c>
       <c r="E22" s="33" t="n">
-        <v>14884</v>
+        <v>14741</v>
       </c>
       <c r="F22" s="33" t="n">
         <v>34.2</v>
@@ -6282,16 +6282,16 @@
         <v>0</v>
       </c>
       <c r="J22" s="33" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K22" s="33" t="n">
-        <v>0</v>
+        <v>143</v>
       </c>
       <c r="L22" s="33" t="n">
-        <v>34.2</v>
+        <v>34.8</v>
       </c>
       <c r="M22" s="33" t="n">
-        <v>7728</v>
+        <v>7871</v>
       </c>
       <c r="N22" s="34" t="inlineStr">
         <is>
@@ -6526,34 +6526,34 @@
         <v>43076</v>
       </c>
       <c r="D23" s="33" t="n">
-        <v>31.6</v>
+        <v>31.2</v>
       </c>
       <c r="E23" s="33" t="n">
-        <v>13618</v>
+        <v>13432</v>
       </c>
       <c r="F23" s="33" t="n">
-        <v>55.5</v>
+        <v>55.1</v>
       </c>
       <c r="G23" s="33" t="n">
-        <v>23900</v>
+        <v>23715</v>
       </c>
       <c r="H23" s="33" t="n">
-        <v>12.9</v>
+        <v>6</v>
       </c>
       <c r="I23" s="33" t="n">
-        <v>5558</v>
+        <v>2594</v>
       </c>
       <c r="J23" s="33" t="n">
-        <v>0</v>
+        <v>7.7</v>
       </c>
       <c r="K23" s="33" t="n">
-        <v>0</v>
+        <v>3335</v>
       </c>
       <c r="L23" s="33" t="n">
-        <v>68.40000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="M23" s="33" t="n">
-        <v>29458</v>
+        <v>29644</v>
       </c>
       <c r="N23" s="34" t="inlineStr">
         <is>
@@ -6800,16 +6800,16 @@
         <v>17399</v>
       </c>
       <c r="H24" s="33" t="n">
-        <v>5.7</v>
+        <v>3.8</v>
       </c>
       <c r="I24" s="33" t="n">
-        <v>1535</v>
+        <v>1023</v>
       </c>
       <c r="J24" s="33" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="K24" s="33" t="n">
-        <v>0</v>
+        <v>512</v>
       </c>
       <c r="L24" s="33" t="n">
         <v>69.8</v>
@@ -7302,34 +7302,34 @@
         <v>75958</v>
       </c>
       <c r="D26" s="33" t="n">
-        <v>51.8</v>
+        <v>51.7</v>
       </c>
       <c r="E26" s="33" t="n">
-        <v>39368</v>
+        <v>39277</v>
       </c>
       <c r="F26" s="33" t="n">
-        <v>42.4</v>
+        <v>41.9</v>
       </c>
       <c r="G26" s="33" t="n">
-        <v>32186</v>
+        <v>31859</v>
       </c>
       <c r="H26" s="33" t="n">
-        <v>5.8</v>
+        <v>4.6</v>
       </c>
       <c r="I26" s="33" t="n">
-        <v>4404</v>
+        <v>3466</v>
       </c>
       <c r="J26" s="33" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="K26" s="33" t="n">
-        <v>0</v>
+        <v>1356</v>
       </c>
       <c r="L26" s="33" t="n">
-        <v>48.2</v>
+        <v>48.3</v>
       </c>
       <c r="M26" s="33" t="n">
-        <v>36590</v>
+        <v>36681</v>
       </c>
       <c r="N26" s="34" t="inlineStr">
         <is>
@@ -7826,10 +7826,10 @@
         <v>56167</v>
       </c>
       <c r="D28" s="33" t="n">
-        <v>13.9</v>
+        <v>13</v>
       </c>
       <c r="E28" s="33" t="n">
-        <v>7801</v>
+        <v>7281</v>
       </c>
       <c r="F28" s="33" t="n">
         <v>83.3</v>
@@ -7838,22 +7838,22 @@
         <v>46806</v>
       </c>
       <c r="H28" s="33" t="n">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
       <c r="I28" s="33" t="n">
-        <v>1560</v>
+        <v>1040</v>
       </c>
       <c r="J28" s="33" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="K28" s="33" t="n">
-        <v>0</v>
+        <v>1040</v>
       </c>
       <c r="L28" s="33" t="n">
-        <v>86.09999999999999</v>
+        <v>87</v>
       </c>
       <c r="M28" s="33" t="n">
-        <v>48366</v>
+        <v>48886</v>
       </c>
       <c r="N28" s="34" t="inlineStr">
         <is>
@@ -8100,16 +8100,16 @@
         <v>14321</v>
       </c>
       <c r="H29" s="33" t="n">
-        <v>6.6</v>
+        <v>4.5</v>
       </c>
       <c r="I29" s="33" t="n">
-        <v>5032</v>
+        <v>3484</v>
       </c>
       <c r="J29" s="33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K29" s="33" t="n">
-        <v>0</v>
+        <v>1548</v>
       </c>
       <c r="L29" s="33" t="n">
         <v>25.3</v>
@@ -8350,10 +8350,10 @@
         <v>371090</v>
       </c>
       <c r="D30" s="33" t="n">
-        <v>58.9</v>
+        <v>58.3</v>
       </c>
       <c r="E30" s="33" t="n">
-        <v>218642</v>
+        <v>216410</v>
       </c>
       <c r="F30" s="33" t="n">
         <v>30.3</v>
@@ -8362,22 +8362,22 @@
         <v>112289</v>
       </c>
       <c r="H30" s="33" t="n">
-        <v>10.8</v>
+        <v>5.7</v>
       </c>
       <c r="I30" s="33" t="n">
-        <v>40159</v>
+        <v>20970</v>
       </c>
       <c r="J30" s="33" t="n">
-        <v>0</v>
+        <v>5.8</v>
       </c>
       <c r="K30" s="33" t="n">
-        <v>0</v>
+        <v>21421</v>
       </c>
       <c r="L30" s="33" t="n">
-        <v>41.1</v>
+        <v>41.7</v>
       </c>
       <c r="M30" s="33" t="n">
-        <v>152448</v>
+        <v>154680</v>
       </c>
       <c r="N30" s="34" t="inlineStr">
         <is>
@@ -8612,10 +8612,10 @@
         <v>83068</v>
       </c>
       <c r="D31" s="33" t="n">
-        <v>62.5</v>
+        <v>61.9</v>
       </c>
       <c r="E31" s="33" t="n">
-        <v>51932</v>
+        <v>51442</v>
       </c>
       <c r="F31" s="33" t="n">
         <v>30</v>
@@ -8630,16 +8630,16 @@
         <v>6176</v>
       </c>
       <c r="J31" s="33" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K31" s="33" t="n">
-        <v>0</v>
+        <v>489</v>
       </c>
       <c r="L31" s="33" t="n">
-        <v>37.5</v>
+        <v>38.1</v>
       </c>
       <c r="M31" s="33" t="n">
-        <v>31136</v>
+        <v>31626</v>
       </c>
       <c r="N31" s="34" t="inlineStr">
         <is>
@@ -8874,10 +8874,10 @@
         <v>86483</v>
       </c>
       <c r="D32" s="33" t="n">
-        <v>58.2</v>
+        <v>57.6</v>
       </c>
       <c r="E32" s="33" t="n">
-        <v>50295</v>
+        <v>49821</v>
       </c>
       <c r="F32" s="33" t="n">
         <v>40.7</v>
@@ -8892,16 +8892,16 @@
         <v>947</v>
       </c>
       <c r="J32" s="33" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K32" s="33" t="n">
-        <v>0</v>
+        <v>474</v>
       </c>
       <c r="L32" s="33" t="n">
-        <v>41.8</v>
+        <v>42.4</v>
       </c>
       <c r="M32" s="33" t="n">
-        <v>36188</v>
+        <v>36662</v>
       </c>
       <c r="N32" s="34" t="inlineStr">
         <is>
@@ -9653,31 +9653,31 @@
         <v>53.7</v>
       </c>
       <c r="E35" s="33" t="n">
-        <v>61948</v>
+        <v>61901</v>
       </c>
       <c r="F35" s="33" t="n">
         <v>41.5</v>
       </c>
       <c r="G35" s="33" t="n">
-        <v>47892</v>
+        <v>47845</v>
       </c>
       <c r="H35" s="33" t="n">
-        <v>4.2</v>
+        <v>3.3</v>
       </c>
       <c r="I35" s="33" t="n">
-        <v>4836</v>
+        <v>3767</v>
       </c>
       <c r="J35" s="33" t="n">
-        <v>0.6</v>
+        <v>1.6</v>
       </c>
       <c r="K35" s="33" t="n">
-        <v>650</v>
+        <v>1812</v>
       </c>
       <c r="L35" s="33" t="n">
         <v>46.3</v>
       </c>
       <c r="M35" s="33" t="n">
-        <v>53378</v>
+        <v>53425</v>
       </c>
       <c r="N35" s="34" t="inlineStr">
         <is>
@@ -9932,10 +9932,10 @@
         <v>79093</v>
       </c>
       <c r="D36" s="33" t="n">
-        <v>61.8</v>
+        <v>61.3</v>
       </c>
       <c r="E36" s="33" t="n">
-        <v>48902</v>
+        <v>48476</v>
       </c>
       <c r="F36" s="33" t="n">
         <v>34.9</v>
@@ -9944,22 +9944,22 @@
         <v>27640</v>
       </c>
       <c r="H36" s="33" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="I36" s="33" t="n">
-        <v>2551</v>
+        <v>1276</v>
       </c>
       <c r="J36" s="33" t="n">
-        <v>0</v>
+        <v>2.2</v>
       </c>
       <c r="K36" s="33" t="n">
-        <v>0</v>
+        <v>1701</v>
       </c>
       <c r="L36" s="33" t="n">
-        <v>38.2</v>
+        <v>38.7</v>
       </c>
       <c r="M36" s="33" t="n">
-        <v>30191</v>
+        <v>30617</v>
       </c>
       <c r="N36" s="34" t="inlineStr">
         <is>
@@ -10194,10 +10194,10 @@
         <v>62616</v>
       </c>
       <c r="D37" s="33" t="n">
-        <v>70.3</v>
+        <v>69.7</v>
       </c>
       <c r="E37" s="33" t="n">
-        <v>44027</v>
+        <v>43655</v>
       </c>
       <c r="F37" s="33" t="n">
         <v>26.8</v>
@@ -10206,22 +10206,22 @@
         <v>16764</v>
       </c>
       <c r="H37" s="33" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="I37" s="33" t="n">
-        <v>1825</v>
+        <v>1645</v>
       </c>
       <c r="J37" s="33" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="K37" s="33" t="n">
-        <v>0</v>
+        <v>551</v>
       </c>
       <c r="L37" s="33" t="n">
-        <v>29.7</v>
+        <v>30.3</v>
       </c>
       <c r="M37" s="33" t="n">
-        <v>18589</v>
+        <v>18961</v>
       </c>
       <c r="N37" s="34" t="inlineStr">
         <is>
@@ -10972,16 +10972,16 @@
         <v>106628</v>
       </c>
       <c r="H40" s="33" t="n">
-        <v>3.2</v>
+        <v>1.8</v>
       </c>
       <c r="I40" s="33" t="n">
-        <v>4898</v>
+        <v>2731</v>
       </c>
       <c r="J40" s="33" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="K40" s="33" t="n">
-        <v>0</v>
+        <v>2167</v>
       </c>
       <c r="L40" s="33" t="n">
         <v>72.90000000000001</v>
@@ -11510,22 +11510,22 @@
         <v>844</v>
       </c>
       <c r="F42" s="33" t="n">
-        <v>87.8</v>
+        <v>87.3</v>
       </c>
       <c r="G42" s="33" t="n">
-        <v>25294</v>
+        <v>25130</v>
       </c>
       <c r="H42" s="33" t="n">
-        <v>9.199999999999999</v>
+        <v>4.7</v>
       </c>
       <c r="I42" s="33" t="n">
-        <v>2659</v>
+        <v>1359</v>
       </c>
       <c r="J42" s="33" t="n">
-        <v>0</v>
+        <v>5.1</v>
       </c>
       <c r="K42" s="33" t="n">
-        <v>0</v>
+        <v>1463</v>
       </c>
       <c r="L42" s="33" t="n">
         <v>97.09999999999999</v>
@@ -11766,10 +11766,10 @@
         <v>194549</v>
       </c>
       <c r="D43" s="33" t="n">
-        <v>38.4</v>
+        <v>37.9</v>
       </c>
       <c r="E43" s="33" t="n">
-        <v>74642</v>
+        <v>73815</v>
       </c>
       <c r="F43" s="33" t="n">
         <v>44.4</v>
@@ -11778,22 +11778,22 @@
         <v>86476</v>
       </c>
       <c r="H43" s="33" t="n">
-        <v>17.2</v>
+        <v>10.7</v>
       </c>
       <c r="I43" s="33" t="n">
-        <v>33431</v>
+        <v>20776</v>
       </c>
       <c r="J43" s="33" t="n">
-        <v>0</v>
+        <v>6.9</v>
       </c>
       <c r="K43" s="33" t="n">
-        <v>0</v>
+        <v>13482</v>
       </c>
       <c r="L43" s="33" t="n">
-        <v>61.6</v>
+        <v>62.1</v>
       </c>
       <c r="M43" s="33" t="n">
-        <v>119907</v>
+        <v>120734</v>
       </c>
       <c r="N43" s="34" t="inlineStr">
         <is>
@@ -12834,10 +12834,10 @@
         <v>6160</v>
       </c>
       <c r="D47" s="33" t="n">
-        <v>73.2</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="E47" s="33" t="n">
-        <v>4509</v>
+        <v>4460</v>
       </c>
       <c r="F47" s="33" t="n">
         <v>20.4</v>
@@ -12846,22 +12846,22 @@
         <v>1257</v>
       </c>
       <c r="H47" s="33" t="n">
-        <v>6.4</v>
+        <v>0</v>
       </c>
       <c r="I47" s="33" t="n">
-        <v>394</v>
+        <v>0</v>
       </c>
       <c r="J47" s="33" t="n">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="K47" s="33" t="n">
-        <v>0</v>
+        <v>444</v>
       </c>
       <c r="L47" s="33" t="n">
-        <v>26.8</v>
+        <v>27.6</v>
       </c>
       <c r="M47" s="33" t="n">
-        <v>1651</v>
+        <v>1700</v>
       </c>
       <c r="N47" s="34" t="inlineStr">
         <is>
@@ -13096,34 +13096,34 @@
         <v>29929</v>
       </c>
       <c r="D48" s="33" t="n">
-        <v>65.09999999999999</v>
+        <v>63.4</v>
       </c>
       <c r="E48" s="33" t="n">
-        <v>19486</v>
+        <v>18976</v>
       </c>
       <c r="F48" s="33" t="n">
-        <v>24.3</v>
+        <v>23.8</v>
       </c>
       <c r="G48" s="33" t="n">
-        <v>7259</v>
+        <v>7132</v>
       </c>
       <c r="H48" s="33" t="n">
-        <v>10.6</v>
+        <v>9.4</v>
       </c>
       <c r="I48" s="33" t="n">
-        <v>3184</v>
+        <v>2802</v>
       </c>
       <c r="J48" s="33" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="K48" s="33" t="n">
-        <v>0</v>
+        <v>1019</v>
       </c>
       <c r="L48" s="33" t="n">
-        <v>34.9</v>
+        <v>36.6</v>
       </c>
       <c r="M48" s="33" t="n">
-        <v>10443</v>
+        <v>10953</v>
       </c>
       <c r="N48" s="34" t="inlineStr">
         <is>
@@ -13348,34 +13348,34 @@
         <v>321096</v>
       </c>
       <c r="D49" s="33" t="n">
-        <v>17.7</v>
+        <v>17</v>
       </c>
       <c r="E49" s="33" t="n">
-        <v>56987</v>
+        <v>54617</v>
       </c>
       <c r="F49" s="33" t="n">
-        <v>76.3</v>
+        <v>76.2</v>
       </c>
       <c r="G49" s="33" t="n">
-        <v>245142</v>
+        <v>244622</v>
       </c>
       <c r="H49" s="33" t="n">
-        <v>5.9</v>
+        <v>4.8</v>
       </c>
       <c r="I49" s="33" t="n">
-        <v>18967</v>
+        <v>15498</v>
       </c>
       <c r="J49" s="33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K49" s="33" t="n">
-        <v>0</v>
+        <v>6359</v>
       </c>
       <c r="L49" s="33" t="n">
-        <v>82.3</v>
+        <v>83</v>
       </c>
       <c r="M49" s="33" t="n">
-        <v>264109</v>
+        <v>266479</v>
       </c>
       <c r="N49" s="34" t="inlineStr">
         <is>
@@ -13600,10 +13600,10 @@
         <v>46949</v>
       </c>
       <c r="D50" s="33" t="n">
-        <v>56.6</v>
+        <v>55.2</v>
       </c>
       <c r="E50" s="33" t="n">
-        <v>26588</v>
+        <v>25915</v>
       </c>
       <c r="F50" s="33" t="n">
         <v>36.2</v>
@@ -13612,22 +13612,22 @@
         <v>16996</v>
       </c>
       <c r="H50" s="33" t="n">
-        <v>6.8</v>
+        <v>5</v>
       </c>
       <c r="I50" s="33" t="n">
-        <v>3197</v>
+        <v>2356</v>
       </c>
       <c r="J50" s="33" t="n">
-        <v>0.4</v>
+        <v>3.6</v>
       </c>
       <c r="K50" s="33" t="n">
-        <v>168</v>
+        <v>1683</v>
       </c>
       <c r="L50" s="33" t="n">
-        <v>43.4</v>
+        <v>44.8</v>
       </c>
       <c r="M50" s="33" t="n">
-        <v>20361</v>
+        <v>21034</v>
       </c>
       <c r="N50" s="34" t="inlineStr">
         <is>
@@ -13852,10 +13852,10 @@
         <v>21140</v>
       </c>
       <c r="D51" s="33" t="n">
-        <v>68.3</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="E51" s="33" t="n">
-        <v>14442</v>
+        <v>14283</v>
       </c>
       <c r="F51" s="33" t="n">
         <v>25.3</v>
@@ -13864,22 +13864,22 @@
         <v>5359</v>
       </c>
       <c r="H51" s="33" t="n">
-        <v>6.3</v>
+        <v>2.6</v>
       </c>
       <c r="I51" s="33" t="n">
-        <v>1340</v>
+        <v>545</v>
       </c>
       <c r="J51" s="33" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="K51" s="33" t="n">
-        <v>0</v>
+        <v>954</v>
       </c>
       <c r="L51" s="33" t="n">
-        <v>31.7</v>
+        <v>32.4</v>
       </c>
       <c r="M51" s="33" t="n">
-        <v>6698</v>
+        <v>6857</v>
       </c>
       <c r="N51" s="34" t="inlineStr">
         <is>
@@ -14104,34 +14104,34 @@
         <v>31281</v>
       </c>
       <c r="D52" s="33" t="n">
-        <v>49.8</v>
+        <v>47.8</v>
       </c>
       <c r="E52" s="33" t="n">
-        <v>15587</v>
+        <v>14947</v>
       </c>
       <c r="F52" s="33" t="n">
-        <v>44.7</v>
+        <v>44.4</v>
       </c>
       <c r="G52" s="33" t="n">
-        <v>13986</v>
+        <v>13879</v>
       </c>
       <c r="H52" s="33" t="n">
-        <v>5.1</v>
+        <v>4.1</v>
       </c>
       <c r="I52" s="33" t="n">
-        <v>1601</v>
+        <v>1281</v>
       </c>
       <c r="J52" s="33" t="n">
-        <v>0.3</v>
+        <v>3.8</v>
       </c>
       <c r="K52" s="33" t="n">
-        <v>107</v>
+        <v>1174</v>
       </c>
       <c r="L52" s="33" t="n">
-        <v>50.2</v>
+        <v>52.2</v>
       </c>
       <c r="M52" s="33" t="n">
-        <v>15694</v>
+        <v>16334</v>
       </c>
       <c r="N52" s="34" t="inlineStr">
         <is>
@@ -14356,10 +14356,10 @@
         <v>48858</v>
       </c>
       <c r="D53" s="33" t="n">
-        <v>67.09999999999999</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="E53" s="33" t="n">
-        <v>32794</v>
+        <v>32461</v>
       </c>
       <c r="F53" s="33" t="n">
         <v>29.7</v>
@@ -14368,22 +14368,22 @@
         <v>14513</v>
       </c>
       <c r="H53" s="33" t="n">
-        <v>3.2</v>
+        <v>2.3</v>
       </c>
       <c r="I53" s="33" t="n">
-        <v>1551</v>
+        <v>1108</v>
       </c>
       <c r="J53" s="33" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="K53" s="33" t="n">
-        <v>0</v>
+        <v>776</v>
       </c>
       <c r="L53" s="33" t="n">
-        <v>32.9</v>
+        <v>33.6</v>
       </c>
       <c r="M53" s="33" t="n">
-        <v>16064</v>
+        <v>16397</v>
       </c>
       <c r="N53" s="34" t="inlineStr">
         <is>
@@ -14608,34 +14608,34 @@
         <v>31931</v>
       </c>
       <c r="D54" s="33" t="n">
-        <v>68.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="E54" s="33" t="n">
-        <v>21832</v>
+        <v>21640</v>
       </c>
       <c r="F54" s="33" t="n">
-        <v>22.6</v>
+        <v>22.3</v>
       </c>
       <c r="G54" s="33" t="n">
-        <v>7213</v>
+        <v>7117</v>
       </c>
       <c r="H54" s="33" t="n">
-        <v>9</v>
+        <v>6.6</v>
       </c>
       <c r="I54" s="33" t="n">
-        <v>2885</v>
+        <v>2116</v>
       </c>
       <c r="J54" s="33" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="K54" s="33" t="n">
-        <v>0</v>
+        <v>1058</v>
       </c>
       <c r="L54" s="33" t="n">
-        <v>31.6</v>
+        <v>32.2</v>
       </c>
       <c r="M54" s="33" t="n">
-        <v>10099</v>
+        <v>10291</v>
       </c>
       <c r="N54" s="34" t="inlineStr">
         <is>
@@ -14860,10 +14860,10 @@
         <v>160918</v>
       </c>
       <c r="D55" s="33" t="n">
-        <v>64.7</v>
+        <v>62.4</v>
       </c>
       <c r="E55" s="33" t="n">
-        <v>104192</v>
+        <v>100333</v>
       </c>
       <c r="F55" s="33" t="n">
         <v>25.7</v>
@@ -14872,22 +14872,22 @@
         <v>41291</v>
       </c>
       <c r="H55" s="33" t="n">
-        <v>9.6</v>
+        <v>6</v>
       </c>
       <c r="I55" s="33" t="n">
-        <v>15436</v>
+        <v>9647</v>
       </c>
       <c r="J55" s="33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K55" s="33" t="n">
-        <v>0</v>
+        <v>9647</v>
       </c>
       <c r="L55" s="33" t="n">
-        <v>35.3</v>
+        <v>37.6</v>
       </c>
       <c r="M55" s="33" t="n">
-        <v>56726</v>
+        <v>60585</v>
       </c>
       <c r="N55" s="34" t="inlineStr">
         <is>
@@ -15364,10 +15364,10 @@
         <v>56819</v>
       </c>
       <c r="D57" s="33" t="n">
-        <v>63.4</v>
+        <v>62.4</v>
       </c>
       <c r="E57" s="33" t="n">
-        <v>36014</v>
+        <v>35440</v>
       </c>
       <c r="F57" s="33" t="n">
         <v>28.3</v>
@@ -15376,22 +15376,22 @@
         <v>16070</v>
       </c>
       <c r="H57" s="33" t="n">
-        <v>8.300000000000001</v>
+        <v>2.5</v>
       </c>
       <c r="I57" s="33" t="n">
-        <v>4735</v>
+        <v>1435</v>
       </c>
       <c r="J57" s="33" t="n">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="K57" s="33" t="n">
-        <v>0</v>
+        <v>3874</v>
       </c>
       <c r="L57" s="33" t="n">
-        <v>36.6</v>
+        <v>37.6</v>
       </c>
       <c r="M57" s="33" t="n">
-        <v>20805</v>
+        <v>21379</v>
       </c>
       <c r="N57" s="34" t="inlineStr">
         <is>
@@ -15616,34 +15616,34 @@
         <v>11326</v>
       </c>
       <c r="D58" s="33" t="n">
-        <v>72.59999999999999</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="E58" s="33" t="n">
-        <v>8218</v>
+        <v>8165</v>
       </c>
       <c r="F58" s="33" t="n">
-        <v>20.5</v>
+        <v>19.5</v>
       </c>
       <c r="G58" s="33" t="n">
-        <v>2318</v>
+        <v>2213</v>
       </c>
       <c r="H58" s="33" t="n">
-        <v>6.5</v>
+        <v>4.7</v>
       </c>
       <c r="I58" s="33" t="n">
-        <v>738</v>
+        <v>527</v>
       </c>
       <c r="J58" s="33" t="n">
-        <v>0.5</v>
+        <v>3.7</v>
       </c>
       <c r="K58" s="33" t="n">
-        <v>53</v>
+        <v>421</v>
       </c>
       <c r="L58" s="33" t="n">
-        <v>27.4</v>
+        <v>27.9</v>
       </c>
       <c r="M58" s="33" t="n">
-        <v>3108</v>
+        <v>3161</v>
       </c>
       <c r="N58" s="34" t="inlineStr">
         <is>
@@ -15868,34 +15868,34 @@
         <v>55986</v>
       </c>
       <c r="D59" s="33" t="n">
-        <v>68.59999999999999</v>
+        <v>68.3</v>
       </c>
       <c r="E59" s="33" t="n">
-        <v>38402</v>
+        <v>38244</v>
       </c>
       <c r="F59" s="33" t="n">
-        <v>24.9</v>
+        <v>24.5</v>
       </c>
       <c r="G59" s="33" t="n">
-        <v>13957</v>
+        <v>13721</v>
       </c>
       <c r="H59" s="33" t="n">
-        <v>6.3</v>
+        <v>3</v>
       </c>
       <c r="I59" s="33" t="n">
-        <v>3548</v>
+        <v>1656</v>
       </c>
       <c r="J59" s="33" t="n">
-        <v>0.1</v>
+        <v>4.2</v>
       </c>
       <c r="K59" s="33" t="n">
-        <v>79</v>
+        <v>2366</v>
       </c>
       <c r="L59" s="33" t="n">
-        <v>31.4</v>
+        <v>31.7</v>
       </c>
       <c r="M59" s="33" t="n">
-        <v>17584</v>
+        <v>17742</v>
       </c>
       <c r="N59" s="34" t="inlineStr">
         <is>
@@ -16144,34 +16144,34 @@
         <v>29679</v>
       </c>
       <c r="D60" s="33" t="n">
-        <v>63.8</v>
+        <v>62.7</v>
       </c>
       <c r="E60" s="33" t="n">
-        <v>18921</v>
+        <v>18616</v>
       </c>
       <c r="F60" s="33" t="n">
-        <v>27.2</v>
+        <v>27</v>
       </c>
       <c r="G60" s="33" t="n">
-        <v>8087</v>
+        <v>8011</v>
       </c>
       <c r="H60" s="33" t="n">
-        <v>9</v>
+        <v>6.2</v>
       </c>
       <c r="I60" s="33" t="n">
-        <v>2670</v>
+        <v>1831</v>
       </c>
       <c r="J60" s="33" t="n">
-        <v>0</v>
+        <v>4.1</v>
       </c>
       <c r="K60" s="33" t="n">
-        <v>0</v>
+        <v>1221</v>
       </c>
       <c r="L60" s="33" t="n">
-        <v>36.2</v>
+        <v>37.3</v>
       </c>
       <c r="M60" s="33" t="n">
-        <v>10758</v>
+        <v>11063</v>
       </c>
       <c r="N60" s="34" t="inlineStr">
         <is>
@@ -16396,10 +16396,10 @@
         <v>246091</v>
       </c>
       <c r="D61" s="33" t="n">
-        <v>56.4</v>
+        <v>55.3</v>
       </c>
       <c r="E61" s="33" t="n">
-        <v>138856</v>
+        <v>136106</v>
       </c>
       <c r="F61" s="33" t="n">
         <v>38.5</v>
@@ -16408,22 +16408,22 @@
         <v>94862</v>
       </c>
       <c r="H61" s="33" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="I61" s="33" t="n">
-        <v>12373</v>
+        <v>10998</v>
       </c>
       <c r="J61" s="33" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="K61" s="33" t="n">
-        <v>0</v>
+        <v>4124</v>
       </c>
       <c r="L61" s="33" t="n">
-        <v>43.6</v>
+        <v>44.7</v>
       </c>
       <c r="M61" s="33" t="n">
-        <v>107235</v>
+        <v>109985</v>
       </c>
       <c r="N61" s="34" t="inlineStr">
         <is>
@@ -16648,34 +16648,34 @@
         <v>49364</v>
       </c>
       <c r="D62" s="33" t="n">
-        <v>68.5</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="E62" s="33" t="n">
-        <v>33817</v>
+        <v>33363</v>
       </c>
       <c r="F62" s="33" t="n">
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="G62" s="33" t="n">
-        <v>12823</v>
+        <v>12596</v>
       </c>
       <c r="H62" s="33" t="n">
-        <v>5.5</v>
+        <v>2.8</v>
       </c>
       <c r="I62" s="33" t="n">
-        <v>2724</v>
+        <v>1362</v>
       </c>
       <c r="J62" s="33" t="n">
-        <v>0</v>
+        <v>4.1</v>
       </c>
       <c r="K62" s="33" t="n">
-        <v>0</v>
+        <v>2043</v>
       </c>
       <c r="L62" s="33" t="n">
-        <v>31.5</v>
+        <v>32.4</v>
       </c>
       <c r="M62" s="33" t="n">
-        <v>15547</v>
+        <v>16001</v>
       </c>
       <c r="N62" s="34" t="inlineStr">
         <is>
@@ -16912,16 +16912,16 @@
         <v>9829</v>
       </c>
       <c r="H63" s="33" t="n">
-        <v>7.5</v>
+        <v>2.4</v>
       </c>
       <c r="I63" s="33" t="n">
-        <v>2837</v>
+        <v>912</v>
       </c>
       <c r="J63" s="33" t="n">
-        <v>0</v>
+        <v>5.1</v>
       </c>
       <c r="K63" s="33" t="n">
-        <v>0</v>
+        <v>1925</v>
       </c>
       <c r="L63" s="33" t="n">
         <v>33.4</v>
@@ -17152,10 +17152,10 @@
         <v>130762</v>
       </c>
       <c r="D64" s="33" t="n">
-        <v>51.6</v>
+        <v>51.3</v>
       </c>
       <c r="E64" s="33" t="n">
-        <v>67511</v>
+        <v>67110</v>
       </c>
       <c r="F64" s="33" t="n">
         <v>46.6</v>
@@ -17164,22 +17164,22 @@
         <v>60949</v>
       </c>
       <c r="H64" s="33" t="n">
-        <v>1.8</v>
+        <v>0.7</v>
       </c>
       <c r="I64" s="33" t="n">
-        <v>2303</v>
+        <v>861</v>
       </c>
       <c r="J64" s="33" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="K64" s="33" t="n">
-        <v>0</v>
+        <v>1842</v>
       </c>
       <c r="L64" s="33" t="n">
-        <v>48.4</v>
+        <v>48.7</v>
       </c>
       <c r="M64" s="33" t="n">
-        <v>63251</v>
+        <v>63652</v>
       </c>
       <c r="N64" s="34" t="inlineStr">
         <is>
@@ -17434,10 +17434,10 @@
         <v>249914</v>
       </c>
       <c r="D65" s="33" t="n">
-        <v>24</v>
+        <v>22.4</v>
       </c>
       <c r="E65" s="33" t="n">
-        <v>59867</v>
+        <v>56105</v>
       </c>
       <c r="F65" s="33" t="n">
         <v>64.59999999999999</v>
@@ -17446,22 +17446,22 @@
         <v>161549</v>
       </c>
       <c r="H65" s="33" t="n">
-        <v>11</v>
+        <v>9.9</v>
       </c>
       <c r="I65" s="33" t="n">
-        <v>27557</v>
+        <v>24735</v>
       </c>
       <c r="J65" s="33" t="n">
-        <v>0.4</v>
+        <v>3</v>
       </c>
       <c r="K65" s="33" t="n">
-        <v>941</v>
+        <v>7526</v>
       </c>
       <c r="L65" s="33" t="n">
-        <v>76</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="M65" s="33" t="n">
-        <v>190047</v>
+        <v>193809</v>
       </c>
       <c r="N65" s="34" t="inlineStr">
         <is>
@@ -17744,16 +17744,16 @@
         <v>7692</v>
       </c>
       <c r="H66" s="33" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="I66" s="33" t="n">
-        <v>398</v>
+        <v>352</v>
       </c>
       <c r="J66" s="33" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="K66" s="33" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="L66" s="33" t="n">
         <v>27.9</v>
@@ -18760,10 +18760,10 @@
         <v>169114</v>
       </c>
       <c r="D70" s="33" t="n">
-        <v>7.2</v>
+        <v>6.4</v>
       </c>
       <c r="E70" s="33" t="n">
-        <v>12175</v>
+        <v>10752</v>
       </c>
       <c r="F70" s="33" t="n">
         <v>60.6</v>
@@ -18772,22 +18772,22 @@
         <v>102498</v>
       </c>
       <c r="H70" s="33" t="n">
-        <v>32.2</v>
+        <v>27.5</v>
       </c>
       <c r="I70" s="33" t="n">
-        <v>54441</v>
+        <v>46583</v>
       </c>
       <c r="J70" s="33" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="K70" s="33" t="n">
-        <v>0</v>
+        <v>9281</v>
       </c>
       <c r="L70" s="33" t="n">
-        <v>92.8</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="M70" s="33" t="n">
-        <v>156939</v>
+        <v>158362</v>
       </c>
       <c r="N70" s="34" t="inlineStr">
         <is>
@@ -19022,34 +19022,34 @@
         <v>328518</v>
       </c>
       <c r="D71" s="33" t="n">
-        <v>23.4</v>
+        <v>22.8</v>
       </c>
       <c r="E71" s="33" t="n">
-        <v>76837</v>
+        <v>74945</v>
       </c>
       <c r="F71" s="33" t="n">
-        <v>72.5</v>
+        <v>72.3</v>
       </c>
       <c r="G71" s="33" t="n">
-        <v>238258</v>
+        <v>237628</v>
       </c>
       <c r="H71" s="33" t="n">
-        <v>4.1</v>
+        <v>1.3</v>
       </c>
       <c r="I71" s="33" t="n">
-        <v>13423</v>
+        <v>4113</v>
       </c>
       <c r="J71" s="33" t="n">
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="K71" s="33" t="n">
-        <v>0</v>
+        <v>11832</v>
       </c>
       <c r="L71" s="33" t="n">
-        <v>76.59999999999999</v>
+        <v>77.2</v>
       </c>
       <c r="M71" s="33" t="n">
-        <v>251681</v>
+        <v>253573</v>
       </c>
       <c r="N71" s="34" t="inlineStr">
         <is>
@@ -19284,10 +19284,10 @@
         <v>91451</v>
       </c>
       <c r="D72" s="33" t="n">
-        <v>41.7</v>
+        <v>41.1</v>
       </c>
       <c r="E72" s="33" t="n">
-        <v>38160</v>
+        <v>37618</v>
       </c>
       <c r="F72" s="33" t="n">
         <v>53.1</v>
@@ -19296,22 +19296,22 @@
         <v>48579</v>
       </c>
       <c r="H72" s="33" t="n">
-        <v>5.1</v>
+        <v>0.7</v>
       </c>
       <c r="I72" s="33" t="n">
-        <v>4701</v>
+        <v>639</v>
       </c>
       <c r="J72" s="33" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K72" s="33" t="n">
-        <v>11</v>
+        <v>4614</v>
       </c>
       <c r="L72" s="33" t="n">
-        <v>58.3</v>
+        <v>58.9</v>
       </c>
       <c r="M72" s="33" t="n">
-        <v>53291</v>
+        <v>53833</v>
       </c>
       <c r="N72" s="34" t="inlineStr">
         <is>
@@ -19546,10 +19546,10 @@
         <v>77814</v>
       </c>
       <c r="D73" s="33" t="n">
-        <v>38.2</v>
+        <v>37.8</v>
       </c>
       <c r="E73" s="33" t="n">
-        <v>29715</v>
+        <v>29442</v>
       </c>
       <c r="F73" s="33" t="n">
         <v>60.2</v>
@@ -19564,16 +19564,16 @@
         <v>934</v>
       </c>
       <c r="J73" s="33" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="K73" s="33" t="n">
-        <v>311</v>
+        <v>585</v>
       </c>
       <c r="L73" s="33" t="n">
-        <v>61.8</v>
+        <v>62.2</v>
       </c>
       <c r="M73" s="33" t="n">
-        <v>48099</v>
+        <v>48372</v>
       </c>
       <c r="N73" s="34" t="inlineStr">
         <is>
@@ -19814,22 +19814,22 @@
         <v>22061</v>
       </c>
       <c r="F74" s="33" t="n">
-        <v>61.5</v>
+        <v>61.2</v>
       </c>
       <c r="G74" s="33" t="n">
-        <v>37530</v>
+        <v>37325</v>
       </c>
       <c r="H74" s="33" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="I74" s="33" t="n">
-        <v>1443</v>
+        <v>987</v>
       </c>
       <c r="J74" s="33" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="K74" s="33" t="n">
-        <v>0</v>
+        <v>661</v>
       </c>
       <c r="L74" s="33" t="n">
         <v>63.9</v>
@@ -20070,34 +20070,34 @@
         <v>51469</v>
       </c>
       <c r="D75" s="33" t="n">
-        <v>23.4</v>
+        <v>22.9</v>
       </c>
       <c r="E75" s="33" t="n">
-        <v>12050</v>
+        <v>11812</v>
       </c>
       <c r="F75" s="33" t="n">
-        <v>73.40000000000001</v>
+        <v>73</v>
       </c>
       <c r="G75" s="33" t="n">
-        <v>37753</v>
+        <v>37594</v>
       </c>
       <c r="H75" s="33" t="n">
-        <v>3.2</v>
+        <v>2.3</v>
       </c>
       <c r="I75" s="33" t="n">
-        <v>1666</v>
+        <v>1189</v>
       </c>
       <c r="J75" s="33" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="K75" s="33" t="n">
-        <v>0</v>
+        <v>874</v>
       </c>
       <c r="L75" s="33" t="n">
-        <v>76.59999999999999</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="M75" s="33" t="n">
-        <v>39419</v>
+        <v>39657</v>
       </c>
       <c r="N75" s="34" t="inlineStr">
         <is>
@@ -20344,16 +20344,16 @@
         <v>17304</v>
       </c>
       <c r="H76" s="33" t="n">
-        <v>10.9</v>
+        <v>10.3</v>
       </c>
       <c r="I76" s="33" t="n">
-        <v>4101</v>
+        <v>3882</v>
       </c>
       <c r="J76" s="33" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K76" s="33" t="n">
-        <v>0</v>
+        <v>219</v>
       </c>
       <c r="L76" s="33" t="n">
         <v>56.7</v>
@@ -20846,10 +20846,10 @@
         <v>40114</v>
       </c>
       <c r="D78" s="33" t="n">
-        <v>36.9</v>
+        <v>36.4</v>
       </c>
       <c r="E78" s="33" t="n">
-        <v>14792</v>
+        <v>14617</v>
       </c>
       <c r="F78" s="33" t="n">
         <v>53.1</v>
@@ -20858,22 +20858,22 @@
         <v>21284</v>
       </c>
       <c r="H78" s="33" t="n">
-        <v>10.1</v>
+        <v>8.6</v>
       </c>
       <c r="I78" s="33" t="n">
-        <v>4039</v>
+        <v>3436</v>
       </c>
       <c r="J78" s="33" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="K78" s="33" t="n">
-        <v>0</v>
+        <v>777</v>
       </c>
       <c r="L78" s="33" t="n">
-        <v>63.1</v>
+        <v>63.6</v>
       </c>
       <c r="M78" s="33" t="n">
-        <v>25322</v>
+        <v>25497</v>
       </c>
       <c r="N78" s="34" t="inlineStr">
         <is>
@@ -21360,10 +21360,10 @@
         <v>66275</v>
       </c>
       <c r="D80" s="33" t="n">
-        <v>61.3</v>
+        <v>60.1</v>
       </c>
       <c r="E80" s="33" t="n">
-        <v>40614</v>
+        <v>39863</v>
       </c>
       <c r="F80" s="33" t="n">
         <v>27.8</v>
@@ -21372,22 +21372,22 @@
         <v>18454</v>
       </c>
       <c r="H80" s="33" t="n">
-        <v>10.9</v>
+        <v>9.4</v>
       </c>
       <c r="I80" s="33" t="n">
-        <v>7207</v>
+        <v>6221</v>
       </c>
       <c r="J80" s="33" t="n">
-        <v>0</v>
+        <v>2.6</v>
       </c>
       <c r="K80" s="33" t="n">
-        <v>0</v>
+        <v>1737</v>
       </c>
       <c r="L80" s="33" t="n">
-        <v>38.7</v>
+        <v>39.9</v>
       </c>
       <c r="M80" s="33" t="n">
-        <v>25661</v>
+        <v>26412</v>
       </c>
       <c r="N80" s="34" t="inlineStr">
         <is>
@@ -21622,16 +21622,16 @@
         <v>91033</v>
       </c>
       <c r="D81" s="33" t="n">
-        <v>40.1</v>
+        <v>39.9</v>
       </c>
       <c r="E81" s="33" t="n">
-        <v>36471</v>
+        <v>36307</v>
       </c>
       <c r="F81" s="33" t="n">
-        <v>56.1</v>
+        <v>55.1</v>
       </c>
       <c r="G81" s="33" t="n">
-        <v>51027</v>
+        <v>50177</v>
       </c>
       <c r="H81" s="33" t="n">
         <v>3.7</v>
@@ -21640,16 +21640,16 @@
         <v>3371</v>
       </c>
       <c r="J81" s="33" t="n">
-        <v>0.2</v>
+        <v>1.3</v>
       </c>
       <c r="K81" s="33" t="n">
-        <v>164</v>
+        <v>1178</v>
       </c>
       <c r="L81" s="33" t="n">
-        <v>59.9</v>
+        <v>60.1</v>
       </c>
       <c r="M81" s="33" t="n">
-        <v>54562</v>
+        <v>54726</v>
       </c>
       <c r="N81" s="34" t="inlineStr">
         <is>
@@ -22146,10 +22146,10 @@
         <v>46289</v>
       </c>
       <c r="D83" s="33" t="n">
-        <v>52.5</v>
+        <v>51.4</v>
       </c>
       <c r="E83" s="33" t="n">
-        <v>24304</v>
+        <v>23770</v>
       </c>
       <c r="F83" s="33" t="n">
         <v>37.6</v>
@@ -22158,22 +22158,22 @@
         <v>17399</v>
       </c>
       <c r="H83" s="33" t="n">
-        <v>9.9</v>
+        <v>9.6</v>
       </c>
       <c r="I83" s="33" t="n">
-        <v>4586</v>
+        <v>4465</v>
       </c>
       <c r="J83" s="33" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="K83" s="33" t="n">
-        <v>0</v>
+        <v>656</v>
       </c>
       <c r="L83" s="33" t="n">
-        <v>47.5</v>
+        <v>48.6</v>
       </c>
       <c r="M83" s="33" t="n">
-        <v>21985</v>
+        <v>22519</v>
       </c>
       <c r="N83" s="34" t="inlineStr">
         <is>
@@ -22408,10 +22408,10 @@
         <v>91986</v>
       </c>
       <c r="D84" s="33" t="n">
-        <v>58.1</v>
+        <v>56.8</v>
       </c>
       <c r="E84" s="33" t="n">
-        <v>53404</v>
+        <v>52259</v>
       </c>
       <c r="F84" s="33" t="n">
         <v>20.2</v>
@@ -22420,22 +22420,22 @@
         <v>18610</v>
       </c>
       <c r="H84" s="33" t="n">
-        <v>21.4</v>
+        <v>15.2</v>
       </c>
       <c r="I84" s="33" t="n">
-        <v>19718</v>
+        <v>13958</v>
       </c>
       <c r="J84" s="33" t="n">
-        <v>0.3</v>
+        <v>7.8</v>
       </c>
       <c r="K84" s="33" t="n">
-        <v>254</v>
+        <v>7159</v>
       </c>
       <c r="L84" s="33" t="n">
-        <v>41.9</v>
+        <v>43.2</v>
       </c>
       <c r="M84" s="33" t="n">
-        <v>38582</v>
+        <v>39727</v>
       </c>
       <c r="N84" s="34" t="inlineStr">
         <is>
@@ -22670,10 +22670,10 @@
         <v>63156</v>
       </c>
       <c r="D85" s="33" t="n">
-        <v>45.3</v>
+        <v>45</v>
       </c>
       <c r="E85" s="33" t="n">
-        <v>28590</v>
+        <v>28391</v>
       </c>
       <c r="F85" s="33" t="n">
         <v>51.1</v>
@@ -22682,22 +22682,22 @@
         <v>32304</v>
       </c>
       <c r="H85" s="33" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
       <c r="I85" s="33" t="n">
-        <v>2263</v>
+        <v>2064</v>
       </c>
       <c r="J85" s="33" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K85" s="33" t="n">
-        <v>0</v>
+        <v>398</v>
       </c>
       <c r="L85" s="33" t="n">
-        <v>54.7</v>
+        <v>55</v>
       </c>
       <c r="M85" s="33" t="n">
-        <v>34566</v>
+        <v>34765</v>
       </c>
       <c r="N85" s="34" t="inlineStr">
         <is>
@@ -23688,10 +23688,10 @@
         <v>160486</v>
       </c>
       <c r="D89" s="33" t="n">
-        <v>45.1</v>
+        <v>45</v>
       </c>
       <c r="E89" s="33" t="n">
-        <v>72442</v>
+        <v>72224</v>
       </c>
       <c r="F89" s="33" t="n">
         <v>52</v>
@@ -23700,22 +23700,22 @@
         <v>83391</v>
       </c>
       <c r="H89" s="33" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="I89" s="33" t="n">
-        <v>4653</v>
+        <v>4132</v>
       </c>
       <c r="J89" s="33" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K89" s="33" t="n">
-        <v>0</v>
+        <v>739</v>
       </c>
       <c r="L89" s="33" t="n">
-        <v>54.9</v>
+        <v>55</v>
       </c>
       <c r="M89" s="33" t="n">
-        <v>88044</v>
+        <v>88262</v>
       </c>
       <c r="N89" s="34" t="inlineStr">
         <is>
@@ -23972,10 +23972,10 @@
         <v>123400</v>
       </c>
       <c r="D90" s="33" t="n">
-        <v>36.1</v>
+        <v>35.5</v>
       </c>
       <c r="E90" s="33" t="n">
-        <v>44576</v>
+        <v>43759</v>
       </c>
       <c r="F90" s="33" t="n">
         <v>55.9</v>
@@ -23984,22 +23984,22 @@
         <v>68993</v>
       </c>
       <c r="H90" s="33" t="n">
-        <v>8</v>
+        <v>7.6</v>
       </c>
       <c r="I90" s="33" t="n">
-        <v>9831</v>
+        <v>9422</v>
       </c>
       <c r="J90" s="33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K90" s="33" t="n">
-        <v>0</v>
+        <v>1226</v>
       </c>
       <c r="L90" s="33" t="n">
-        <v>63.9</v>
+        <v>64.5</v>
       </c>
       <c r="M90" s="33" t="n">
-        <v>78824</v>
+        <v>79641</v>
       </c>
       <c r="N90" s="34" t="inlineStr">
         <is>

</xml_diff>